<commit_message>
Fix employment index cache fallback: y_j join key mismatch
The y_j_output.csv cache stores columns as lowercase Haver codes
(e.g., ustia1), but the fallback path joined on var_name (e.g., farms),
producing 0 matches. This caused empty employment index CSVs, which
made F9/F10 silently drop from the Drupal HTML. Fixed by using the
same haver_code_lower join logic as the Haver-available path.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/publication/tariff_impacts_results_20260326.xlsx
+++ b/output/publication/tariff_impacts_results_20260326.xlsx
@@ -6,7 +6,7 @@
     <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Data TOC" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Data TOC" sheetId="23" state="visible" r:id="rId23"/>
     <sheet name="F1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="F2" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="F3" sheetId="3" state="visible" r:id="rId3"/>
@@ -20,19 +20,21 @@
     <sheet name="F6" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="F7" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="F8" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="F11" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="F12" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="F13" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="F14" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="F15" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="FA2" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="FA3" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="F9" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="F10" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="F11" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="F12" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="F13" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="F14" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="F15" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="FA2" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="FA3" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="225">
   <si>
     <t xml:space="preserve">Figure 1. Daily Effective Tariff Rate (Import-Weighted)</t>
   </si>
@@ -583,6 +585,24 @@
     <t xml:space="preserve">Deviation from trend (%)</t>
   </si>
   <si>
+    <t xml:space="preserve">Figure 9. Tariff-Exposed Employment Index</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subtitle: Leontief-adjusted total import content weighting, index (Dec 2024 = 100)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source: BLS via Haver, USITC DataWeb, BEA I-O Tables (including Total Requirements), and The Budget Lab analysis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Employment index</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Figure 10. Manufacturing Tariff-Exposed Employment Index</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manufacturing employment index</t>
+  </si>
+  <si>
     <t xml:space="preserve">Figure 11. Manufacturing Industrial Production</t>
   </si>
   <si>
@@ -12306,6 +12326,1162 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
+    <col min="1" max="1" width="112.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="16.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="11.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="24.71" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="n">
+        <v>44927</v>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>99.9779164132285</v>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>100.234556485889</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>-0.256039515370743</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="n">
+        <v>44958</v>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>100.036929745838</v>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>100.236901680715</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>-0.199499317640361</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="n">
+        <v>44986</v>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>100.023411816636</v>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>100.239019921203</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>-0.215093987089165</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="n">
+        <v>45017</v>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>100.11116406403</v>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>100.241365116029</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>-0.12988754876655</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="n">
+        <v>45047</v>
+      </c>
+      <c r="B10" s="7" t="n">
+        <v>100.127207973884</v>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>100.243634659409</v>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>-0.116143719171058</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="n">
+        <v>45078</v>
+      </c>
+      <c r="B11" s="7" t="n">
+        <v>100.270493162611</v>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>100.245979854235</v>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>0.0244531585315455</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="n">
+        <v>45108</v>
+      </c>
+      <c r="B12" s="7" t="n">
+        <v>100.273192294655</v>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>100.248249397615</v>
+      </c>
+      <c r="D12" s="7" t="n">
+        <v>0.0248811297847373</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="n">
+        <v>45139</v>
+      </c>
+      <c r="B13" s="7" t="n">
+        <v>100.373611002875</v>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>100.250594592441</v>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>0.122708908544689</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="n">
+        <v>45170</v>
+      </c>
+      <c r="B14" s="7" t="n">
+        <v>100.431679379832</v>
+      </c>
+      <c r="C14" s="7" t="n">
+        <v>100.252939787267</v>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>0.178288629683898</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="n">
+        <v>45200</v>
+      </c>
+      <c r="B15" s="7" t="n">
+        <v>100.304967898637</v>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>100.255209330648</v>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>0.0496319027426528</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="n">
+        <v>45231</v>
+      </c>
+      <c r="B16" s="7" t="n">
+        <v>100.456676454201</v>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>100.257554525474</v>
+      </c>
+      <c r="D16" s="7" t="n">
+        <v>0.198610398657295</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="n">
+        <v>45261</v>
+      </c>
+      <c r="B17" s="7" t="n">
+        <v>100.505622041725</v>
+      </c>
+      <c r="C17" s="7" t="n">
+        <v>100.259824068854</v>
+      </c>
+      <c r="D17" s="7" t="n">
+        <v>0.245160985623083</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="n">
+        <v>45292</v>
+      </c>
+      <c r="B18" s="7" t="n">
+        <v>100.452971935306</v>
+      </c>
+      <c r="C18" s="7" t="n">
+        <v>100.26216926368</v>
+      </c>
+      <c r="D18" s="7" t="n">
+        <v>0.190303753676413</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="n">
+        <v>45323</v>
+      </c>
+      <c r="B19" s="7" t="n">
+        <v>100.426475188889</v>
+      </c>
+      <c r="C19" s="7" t="n">
+        <v>100.264514458506</v>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>0.161533451050055</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="n">
+        <v>45352</v>
+      </c>
+      <c r="B20" s="7" t="n">
+        <v>100.419093000354</v>
+      </c>
+      <c r="C20" s="7" t="n">
+        <v>100.26670835044</v>
+      </c>
+      <c r="D20" s="7" t="n">
+        <v>0.151979308407668</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="n">
+        <v>45383</v>
+      </c>
+      <c r="B21" s="7" t="n">
+        <v>100.479238339088</v>
+      </c>
+      <c r="C21" s="7" t="n">
+        <v>100.269053545266</v>
+      </c>
+      <c r="D21" s="7" t="n">
+        <v>0.209620801623323</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="n">
+        <v>45413</v>
+      </c>
+      <c r="B22" s="7" t="n">
+        <v>100.461171720553</v>
+      </c>
+      <c r="C22" s="7" t="n">
+        <v>100.271323088646</v>
+      </c>
+      <c r="D22" s="7" t="n">
+        <v>0.189334922547402</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="n">
+        <v>45444</v>
+      </c>
+      <c r="B23" s="7" t="n">
+        <v>100.418652853807</v>
+      </c>
+      <c r="C23" s="7" t="n">
+        <v>100.273668283472</v>
+      </c>
+      <c r="D23" s="7" t="n">
+        <v>0.144588876438756</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="n">
+        <v>45474</v>
+      </c>
+      <c r="B24" s="7" t="n">
+        <v>100.385717628962</v>
+      </c>
+      <c r="C24" s="7" t="n">
+        <v>100.275937826852</v>
+      </c>
+      <c r="D24" s="7" t="n">
+        <v>0.109477711691097</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="n">
+        <v>45505</v>
+      </c>
+      <c r="B25" s="7" t="n">
+        <v>100.194151604928</v>
+      </c>
+      <c r="C25" s="7" t="n">
+        <v>100.278283021678</v>
+      </c>
+      <c r="D25" s="7" t="n">
+        <v>-0.0838979430190512</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="n">
+        <v>45536</v>
+      </c>
+      <c r="B26" s="7" t="n">
+        <v>100.186574849697</v>
+      </c>
+      <c r="C26" s="7" t="n">
+        <v>100.280628216504</v>
+      </c>
+      <c r="D26" s="7" t="n">
+        <v>-0.0937901651391848</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="n">
+        <v>45566</v>
+      </c>
+      <c r="B27" s="7" t="n">
+        <v>99.8817196846808</v>
+      </c>
+      <c r="C27" s="7" t="n">
+        <v>100.282897759884</v>
+      </c>
+      <c r="D27" s="7" t="n">
+        <v>-0.400046353032191</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="n">
+        <v>45597</v>
+      </c>
+      <c r="B28" s="7" t="n">
+        <v>100.065129633092</v>
+      </c>
+      <c r="C28" s="7" t="n">
+        <v>100.28524295471</v>
+      </c>
+      <c r="D28" s="7" t="n">
+        <v>-0.219487249701822</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="12" t="n">
+        <v>45627</v>
+      </c>
+      <c r="B29" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="C29" s="7" t="n">
+        <v>100.28751249809</v>
+      </c>
+      <c r="D29" s="7" t="n">
+        <v>-0.286688233588206</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="12" t="n">
+        <v>45658</v>
+      </c>
+      <c r="B30" s="7" t="n">
+        <v>99.7592491839363</v>
+      </c>
+      <c r="C30" s="7" t="n">
+        <v>100.289857692916</v>
+      </c>
+      <c r="D30" s="7" t="n">
+        <v>-0.529074944552022</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="n">
+        <v>45689</v>
+      </c>
+      <c r="B31" s="7" t="n">
+        <v>99.8082166498581</v>
+      </c>
+      <c r="C31" s="7" t="n">
+        <v>100.292202887742</v>
+      </c>
+      <c r="D31" s="7" t="n">
+        <v>-0.482576136477997</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="n">
+        <v>45717</v>
+      </c>
+      <c r="B32" s="7" t="n">
+        <v>99.8067115743737</v>
+      </c>
+      <c r="C32" s="7" t="n">
+        <v>100.29432112823</v>
+      </c>
+      <c r="D32" s="7" t="n">
+        <v>-0.486178627435319</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="12" t="n">
+        <v>45748</v>
+      </c>
+      <c r="B33" s="7" t="n">
+        <v>99.8889287534598</v>
+      </c>
+      <c r="C33" s="7" t="n">
+        <v>100.296666323057</v>
+      </c>
+      <c r="D33" s="7" t="n">
+        <v>-0.406531527462151</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="12" t="n">
+        <v>45778</v>
+      </c>
+      <c r="B34" s="7" t="n">
+        <v>99.8478157382411</v>
+      </c>
+      <c r="C34" s="7" t="n">
+        <v>100.298935866437</v>
+      </c>
+      <c r="D34" s="7" t="n">
+        <v>-0.449775587645551</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="n">
+        <v>45809</v>
+      </c>
+      <c r="B35" s="7" t="n">
+        <v>99.7882607379367</v>
+      </c>
+      <c r="C35" s="7" t="n">
+        <v>100.301281061263</v>
+      </c>
+      <c r="D35" s="7" t="n">
+        <v>-0.51147933296346</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="12" t="n">
+        <v>45839</v>
+      </c>
+      <c r="B36" s="7" t="n">
+        <v>99.7424512641067</v>
+      </c>
+      <c r="C36" s="7" t="n">
+        <v>100.303550604643</v>
+      </c>
+      <c r="D36" s="7" t="n">
+        <v>-0.55940127458467</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="12" t="n">
+        <v>45870</v>
+      </c>
+      <c r="B37" s="7" t="n">
+        <v>99.6544680946629</v>
+      </c>
+      <c r="C37" s="7" t="n">
+        <v>100.305895799469</v>
+      </c>
+      <c r="D37" s="7" t="n">
+        <v>-0.649441091786074</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="12" t="n">
+        <v>45901</v>
+      </c>
+      <c r="B38" s="7" t="n">
+        <v>99.6687423220202</v>
+      </c>
+      <c r="C38" s="7" t="n">
+        <v>100.308240994295</v>
+      </c>
+      <c r="D38" s="7" t="n">
+        <v>-0.637533532574808</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="12" t="n">
+        <v>45931</v>
+      </c>
+      <c r="B39" s="7" t="n">
+        <v>99.6643127751522</v>
+      </c>
+      <c r="C39" s="7" t="n">
+        <v>100.310510537675</v>
+      </c>
+      <c r="D39" s="7" t="n">
+        <v>-0.644197461521179</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="12" t="n">
+        <v>45962</v>
+      </c>
+      <c r="B40" s="7" t="n">
+        <v>99.6631849629043</v>
+      </c>
+      <c r="C40" s="7" t="n">
+        <v>100.312855732501</v>
+      </c>
+      <c r="D40" s="7" t="n">
+        <v>-0.647644576413087</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="12" t="n">
+        <v>45992</v>
+      </c>
+      <c r="B41" s="7" t="n">
+        <v>99.6000041885583</v>
+      </c>
+      <c r="C41" s="7" t="n">
+        <v>100.315125275881</v>
+      </c>
+      <c r="D41" s="7" t="n">
+        <v>-0.712874639149386</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="12" t="n">
+        <v>46023</v>
+      </c>
+      <c r="B42" s="7" t="n">
+        <v>99.6333176941297</v>
+      </c>
+      <c r="C42" s="7" t="n">
+        <v>100.317470470707</v>
+      </c>
+      <c r="D42" s="7" t="n">
+        <v>-0.681987667120354</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="13" t="n">
+        <v>46054</v>
+      </c>
+      <c r="B43" s="11" t="n">
+        <v>99.4457248047046</v>
+      </c>
+      <c r="C43" s="11" t="n">
+        <v>100.319815665533</v>
+      </c>
+      <c r="D43" s="11" t="n">
+        <v>-0.871304293204411</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="112.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="30.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="11.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="24.71" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="n">
+        <v>44927</v>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>101.975907993689</v>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>102.221441072174</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>-0.24019723837756</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="n">
+        <v>44958</v>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>101.890646715014</v>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>102.141689170622</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>-0.245778641068872</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="n">
+        <v>44986</v>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>101.860071986868</v>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>102.069655195026</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>-0.2053335124513</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="n">
+        <v>45017</v>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>101.820535800949</v>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>101.989903293474</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>-0.166062999430294</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="n">
+        <v>45047</v>
+      </c>
+      <c r="B10" s="7" t="n">
+        <v>101.700845049265</v>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>101.912724033908</v>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>-0.207902385743342</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="n">
+        <v>45078</v>
+      </c>
+      <c r="B11" s="7" t="n">
+        <v>101.78553588737</v>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>101.832972132355</v>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>-0.0465824025285499</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="n">
+        <v>45108</v>
+      </c>
+      <c r="B12" s="7" t="n">
+        <v>101.71065428921</v>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>101.755792872789</v>
+      </c>
+      <c r="D12" s="7" t="n">
+        <v>-0.0443597187975375</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="n">
+        <v>45139</v>
+      </c>
+      <c r="B13" s="7" t="n">
+        <v>101.75453442914</v>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>101.676040971236</v>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>0.0771995616217325</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="n">
+        <v>45170</v>
+      </c>
+      <c r="B14" s="7" t="n">
+        <v>101.802333195414</v>
+      </c>
+      <c r="C14" s="7" t="n">
+        <v>101.596289069684</v>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>0.202806743845452</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="n">
+        <v>45200</v>
+      </c>
+      <c r="B15" s="7" t="n">
+        <v>101.403830662819</v>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>101.519109810117</v>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>-0.113554135289406</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="n">
+        <v>45231</v>
+      </c>
+      <c r="B16" s="7" t="n">
+        <v>101.648564918326</v>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>101.439357908565</v>
+      </c>
+      <c r="D16" s="7" t="n">
+        <v>0.206238499606615</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="n">
+        <v>45261</v>
+      </c>
+      <c r="B17" s="7" t="n">
+        <v>101.744655325218</v>
+      </c>
+      <c r="C17" s="7" t="n">
+        <v>101.362178648999</v>
+      </c>
+      <c r="D17" s="7" t="n">
+        <v>0.377336676576046</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="n">
+        <v>45292</v>
+      </c>
+      <c r="B18" s="7" t="n">
+        <v>101.718206633141</v>
+      </c>
+      <c r="C18" s="7" t="n">
+        <v>101.282426747446</v>
+      </c>
+      <c r="D18" s="7" t="n">
+        <v>0.430262089573663</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="n">
+        <v>45323</v>
+      </c>
+      <c r="B19" s="7" t="n">
+        <v>101.524599455771</v>
+      </c>
+      <c r="C19" s="7" t="n">
+        <v>101.202674845894</v>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>0.318098914250631</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="n">
+        <v>45352</v>
+      </c>
+      <c r="B20" s="7" t="n">
+        <v>101.356168963816</v>
+      </c>
+      <c r="C20" s="7" t="n">
+        <v>101.128068228313</v>
+      </c>
+      <c r="D20" s="7" t="n">
+        <v>0.225556306472918</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="n">
+        <v>45383</v>
+      </c>
+      <c r="B21" s="7" t="n">
+        <v>101.349715168125</v>
+      </c>
+      <c r="C21" s="7" t="n">
+        <v>101.048316326761</v>
+      </c>
+      <c r="D21" s="7" t="n">
+        <v>0.298272007214129</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="n">
+        <v>45413</v>
+      </c>
+      <c r="B22" s="7" t="n">
+        <v>101.268780101682</v>
+      </c>
+      <c r="C22" s="7" t="n">
+        <v>100.971137067194</v>
+      </c>
+      <c r="D22" s="7" t="n">
+        <v>0.294780313596155</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="n">
+        <v>45444</v>
+      </c>
+      <c r="B23" s="7" t="n">
+        <v>101.101929354924</v>
+      </c>
+      <c r="C23" s="7" t="n">
+        <v>100.891385165642</v>
+      </c>
+      <c r="D23" s="7" t="n">
+        <v>0.208684010965832</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="n">
+        <v>45474</v>
+      </c>
+      <c r="B24" s="7" t="n">
+        <v>101.019454185154</v>
+      </c>
+      <c r="C24" s="7" t="n">
+        <v>100.814205906075</v>
+      </c>
+      <c r="D24" s="7" t="n">
+        <v>0.203590632128248</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="n">
+        <v>45505</v>
+      </c>
+      <c r="B25" s="7" t="n">
+        <v>100.646656309727</v>
+      </c>
+      <c r="C25" s="7" t="n">
+        <v>100.734454004523</v>
+      </c>
+      <c r="D25" s="7" t="n">
+        <v>-0.0871575625868148</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="n">
+        <v>45536</v>
+      </c>
+      <c r="B26" s="7" t="n">
+        <v>100.539173355552</v>
+      </c>
+      <c r="C26" s="7" t="n">
+        <v>100.654702102971</v>
+      </c>
+      <c r="D26" s="7" t="n">
+        <v>-0.114777298034385</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="n">
+        <v>45566</v>
+      </c>
+      <c r="B27" s="7" t="n">
+        <v>99.9313285803689</v>
+      </c>
+      <c r="C27" s="7" t="n">
+        <v>100.577522843404</v>
+      </c>
+      <c r="D27" s="7" t="n">
+        <v>-0.64248377248366</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="n">
+        <v>45597</v>
+      </c>
+      <c r="B28" s="7" t="n">
+        <v>100.186281679762</v>
+      </c>
+      <c r="C28" s="7" t="n">
+        <v>100.497770941852</v>
+      </c>
+      <c r="D28" s="7" t="n">
+        <v>-0.309946438781705</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="12" t="n">
+        <v>45627</v>
+      </c>
+      <c r="B29" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="C29" s="7" t="n">
+        <v>100.420591682285</v>
+      </c>
+      <c r="D29" s="7" t="n">
+        <v>-0.418830117647184</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="12" t="n">
+        <v>45658</v>
+      </c>
+      <c r="B30" s="7" t="n">
+        <v>99.8146492880884</v>
+      </c>
+      <c r="C30" s="7" t="n">
+        <v>100.340839780733</v>
+      </c>
+      <c r="D30" s="7" t="n">
+        <v>-0.524403118205974</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="n">
+        <v>45689</v>
+      </c>
+      <c r="B31" s="7" t="n">
+        <v>99.8179046115021</v>
+      </c>
+      <c r="C31" s="7" t="n">
+        <v>100.26108787918</v>
+      </c>
+      <c r="D31" s="7" t="n">
+        <v>-0.442029183058912</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="n">
+        <v>45717</v>
+      </c>
+      <c r="B32" s="7" t="n">
+        <v>99.7644666402592</v>
+      </c>
+      <c r="C32" s="7" t="n">
+        <v>100.189053903585</v>
+      </c>
+      <c r="D32" s="7" t="n">
+        <v>-0.423786079200061</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="12" t="n">
+        <v>45748</v>
+      </c>
+      <c r="B33" s="7" t="n">
+        <v>99.7362896741851</v>
+      </c>
+      <c r="C33" s="7" t="n">
+        <v>100.109302002033</v>
+      </c>
+      <c r="D33" s="7" t="n">
+        <v>-0.372605063053943</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="12" t="n">
+        <v>45778</v>
+      </c>
+      <c r="B34" s="7" t="n">
+        <v>99.629339633489</v>
+      </c>
+      <c r="C34" s="7" t="n">
+        <v>100.032122742466</v>
+      </c>
+      <c r="D34" s="7" t="n">
+        <v>-0.402653765544725</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="n">
+        <v>45809</v>
+      </c>
+      <c r="B35" s="7" t="n">
+        <v>99.5199744471928</v>
+      </c>
+      <c r="C35" s="7" t="n">
+        <v>99.9523708409137</v>
+      </c>
+      <c r="D35" s="7" t="n">
+        <v>-0.432602438624596</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="12" t="n">
+        <v>45839</v>
+      </c>
+      <c r="B36" s="7" t="n">
+        <v>99.4339691892635</v>
+      </c>
+      <c r="C36" s="7" t="n">
+        <v>99.875191581347</v>
+      </c>
+      <c r="D36" s="7" t="n">
+        <v>-0.44177376293103</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="12" t="n">
+        <v>45870</v>
+      </c>
+      <c r="B37" s="7" t="n">
+        <v>99.3082596052685</v>
+      </c>
+      <c r="C37" s="7" t="n">
+        <v>99.7954396797947</v>
+      </c>
+      <c r="D37" s="7" t="n">
+        <v>-0.488178694426755</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="12" t="n">
+        <v>45901</v>
+      </c>
+      <c r="B38" s="7" t="n">
+        <v>99.2938469319734</v>
+      </c>
+      <c r="C38" s="7" t="n">
+        <v>99.7156877782425</v>
+      </c>
+      <c r="D38" s="7" t="n">
+        <v>-0.423043610958407</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="12" t="n">
+        <v>45931</v>
+      </c>
+      <c r="B39" s="7" t="n">
+        <v>99.2278590387136</v>
+      </c>
+      <c r="C39" s="7" t="n">
+        <v>99.6385085186758</v>
+      </c>
+      <c r="D39" s="7" t="n">
+        <v>-0.412139328525951</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="12" t="n">
+        <v>45962</v>
+      </c>
+      <c r="B40" s="7" t="n">
+        <v>99.1712739693549</v>
+      </c>
+      <c r="C40" s="7" t="n">
+        <v>99.5587566171235</v>
+      </c>
+      <c r="D40" s="7" t="n">
+        <v>-0.389199966868625</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="12" t="n">
+        <v>45992</v>
+      </c>
+      <c r="B41" s="7" t="n">
+        <v>99.0906911856667</v>
+      </c>
+      <c r="C41" s="7" t="n">
+        <v>99.4815773575569</v>
+      </c>
+      <c r="D41" s="7" t="n">
+        <v>-0.392923174594684</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="12" t="n">
+        <v>46023</v>
+      </c>
+      <c r="B42" s="7" t="n">
+        <v>99.1451576482527</v>
+      </c>
+      <c r="C42" s="7" t="n">
+        <v>99.4018254560046</v>
+      </c>
+      <c r="D42" s="7" t="n">
+        <v>-0.258212368409172</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="13" t="n">
+        <v>46054</v>
+      </c>
+      <c r="B43" s="11" t="n">
+        <v>99.0825044206099</v>
+      </c>
+      <c r="C43" s="11" t="n">
+        <v>99.3220735544524</v>
+      </c>
+      <c r="D43" s="11" t="n">
+        <v>-0.24120432172724</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
     <col min="1" max="1" width="70.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="27.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="11.71" hidden="0" customWidth="1"/>
@@ -12314,17 +13490,17 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
     </row>
     <row r="5">
@@ -12332,7 +13508,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>181</v>
@@ -13215,7 +14391,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
@@ -13229,17 +14405,17 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
     </row>
     <row r="5">
@@ -13247,16 +14423,16 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
     </row>
     <row r="6">
@@ -27409,7 +28585,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
@@ -27425,17 +28601,17 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
     </row>
     <row r="5">
@@ -27443,22 +28619,22 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
     </row>
     <row r="6">
@@ -28318,7 +29494,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
@@ -28334,17 +29510,17 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
     </row>
     <row r="5">
@@ -28352,22 +29528,22 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
     </row>
     <row r="6">
@@ -29219,1548 +30395,6 @@
       </c>
       <c r="G42" s="11" t="n">
         <v>4.59008748746008</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
-  <cols>
-    <col min="1" max="1" width="80.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="12.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="13.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="26.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="29.71" hidden="0" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>197</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>198</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>207</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="12" t="n">
-        <v>45627</v>
-      </c>
-      <c r="B6" s="7" t="n">
-        <v>253703</v>
-      </c>
-      <c r="C6" s="7" t="n">
-        <v>243438.774684143</v>
-      </c>
-      <c r="D6" s="7" t="n">
-        <v>11.7687358107597</v>
-      </c>
-      <c r="E6" s="7" t="n">
-        <v>11.7687358107597</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="12" t="n">
-        <v>45658</v>
-      </c>
-      <c r="B7" s="7" t="n">
-        <v>285683</v>
-      </c>
-      <c r="C7" s="7" t="n">
-        <v>244374.646013476</v>
-      </c>
-      <c r="D7" s="7" t="n">
-        <v>47.3632534248561</v>
-      </c>
-      <c r="E7" s="7" t="n">
-        <v>59.1319892356158</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="12" t="n">
-        <v>45689</v>
-      </c>
-      <c r="B8" s="7" t="n">
-        <v>282954</v>
-      </c>
-      <c r="C8" s="7" t="n">
-        <v>245310.517342808</v>
-      </c>
-      <c r="D8" s="7" t="n">
-        <v>43.1611922728362</v>
-      </c>
-      <c r="E8" s="7" t="n">
-        <v>102.293181508452</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="12" t="n">
-        <v>45717</v>
-      </c>
-      <c r="B9" s="7" t="n">
-        <v>300358</v>
-      </c>
-      <c r="C9" s="7" t="n">
-        <v>246155.820478979</v>
-      </c>
-      <c r="D9" s="7" t="n">
-        <v>62.1470312196687</v>
-      </c>
-      <c r="E9" s="7" t="n">
-        <v>164.440212728121</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="12" t="n">
-        <v>45748</v>
-      </c>
-      <c r="B10" s="7" t="n">
-        <v>240461</v>
-      </c>
-      <c r="C10" s="7" t="n">
-        <v>247091.691808312</v>
-      </c>
-      <c r="D10" s="7" t="n">
-        <v>-7.60260591844516</v>
-      </c>
-      <c r="E10" s="7" t="n">
-        <v>156.837606809676</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="12" t="n">
-        <v>45778</v>
-      </c>
-      <c r="B11" s="7" t="n">
-        <v>241089</v>
-      </c>
-      <c r="C11" s="7" t="n">
-        <v>247997.373739924</v>
-      </c>
-      <c r="D11" s="7" t="n">
-        <v>-7.92098993594275</v>
-      </c>
-      <c r="E11" s="7" t="n">
-        <v>148.916616873733</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="12" t="n">
-        <v>45809</v>
-      </c>
-      <c r="B12" s="7" t="n">
-        <v>230650</v>
-      </c>
-      <c r="C12" s="7" t="n">
-        <v>248933.245069256</v>
-      </c>
-      <c r="D12" s="7" t="n">
-        <v>-20.9631681263894</v>
-      </c>
-      <c r="E12" s="7" t="n">
-        <v>127.953448747343</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="12" t="n">
-        <v>45839</v>
-      </c>
-      <c r="B13" s="7" t="n">
-        <v>245921</v>
-      </c>
-      <c r="C13" s="7" t="n">
-        <v>249838.927000868</v>
-      </c>
-      <c r="D13" s="7" t="n">
-        <v>-4.49220923938841</v>
-      </c>
-      <c r="E13" s="7" t="n">
-        <v>123.461239507955</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="12" t="n">
-        <v>45870</v>
-      </c>
-      <c r="B14" s="7" t="n">
-        <v>229128</v>
-      </c>
-      <c r="C14" s="7" t="n">
-        <v>250774.7983302</v>
-      </c>
-      <c r="D14" s="7" t="n">
-        <v>-24.8197445844608</v>
-      </c>
-      <c r="E14" s="7" t="n">
-        <v>98.6414949234942</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="12" t="n">
-        <v>45901</v>
-      </c>
-      <c r="B15" s="7" t="n">
-        <v>231589</v>
-      </c>
-      <c r="C15" s="7" t="n">
-        <v>251710.669659533</v>
-      </c>
-      <c r="D15" s="7" t="n">
-        <v>-23.0710654732595</v>
-      </c>
-      <c r="E15" s="7" t="n">
-        <v>75.5704294502347</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="12" t="n">
-        <v>45931</v>
-      </c>
-      <c r="B16" s="7" t="n">
-        <v>221136</v>
-      </c>
-      <c r="C16" s="7" t="n">
-        <v>252616.351591145</v>
-      </c>
-      <c r="D16" s="7" t="n">
-        <v>-36.0946812550641</v>
-      </c>
-      <c r="E16" s="7" t="n">
-        <v>39.4757481951706</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="12" t="n">
-        <v>45962</v>
-      </c>
-      <c r="B17" s="7" t="n">
-        <v>233624</v>
-      </c>
-      <c r="C17" s="7" t="n">
-        <v>253552.222920477</v>
-      </c>
-      <c r="D17" s="7" t="n">
-        <v>-22.8492636815663</v>
-      </c>
-      <c r="E17" s="7" t="n">
-        <v>16.6264845136043</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="12" t="n">
-        <v>45992</v>
-      </c>
-      <c r="B18" s="7" t="n">
-        <v>242150</v>
-      </c>
-      <c r="C18" s="7" t="n">
-        <v>254457.904852089</v>
-      </c>
-      <c r="D18" s="7" t="n">
-        <v>-14.111973980582</v>
-      </c>
-      <c r="E18" s="7" t="n">
-        <v>2.51451053302223</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="13" t="n">
-        <v>46023</v>
-      </c>
-      <c r="B19" s="11" t="n">
-        <v>238920</v>
-      </c>
-      <c r="C19" s="11" t="n">
-        <v>255393.776181421</v>
-      </c>
-      <c r="D19" s="11" t="n">
-        <v>-18.8884707533868</v>
-      </c>
-      <c r="E19" s="11" t="n">
-        <v>-16.3739602203646</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
-  <cols>
-    <col min="1" max="1" width="86.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="16.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="29.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="29.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="29.71" hidden="0" customWidth="1"/>
-    <col min="6" max="6" width="19.71" hidden="0" customWidth="1"/>
-    <col min="7" max="7" width="32.71" hidden="0" customWidth="1"/>
-    <col min="8" max="8" width="32.71" hidden="0" customWidth="1"/>
-    <col min="9" max="9" width="32.71" hidden="0" customWidth="1"/>
-    <col min="10" max="10" width="18.71" hidden="0" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>211</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>212</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="12" t="n">
-        <v>44927</v>
-      </c>
-      <c r="B6" s="7" t="n">
-        <v>100.693736917178</v>
-      </c>
-      <c r="C6" s="7" t="n">
-        <v>100.92968518895</v>
-      </c>
-      <c r="D6" s="7" t="n">
-        <v>100.601424908979</v>
-      </c>
-      <c r="E6" s="7" t="n">
-        <v>101.259016575136</v>
-      </c>
-      <c r="F6" s="7" t="n">
-        <v>103.849235112349</v>
-      </c>
-      <c r="G6" s="7" t="n">
-        <v>104.193354593693</v>
-      </c>
-      <c r="H6" s="7" t="n">
-        <v>103.694733127383</v>
-      </c>
-      <c r="I6" s="7" t="n">
-        <v>104.694373707011</v>
-      </c>
-      <c r="J6" s="6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="12" t="n">
-        <v>44958</v>
-      </c>
-      <c r="B7" s="7" t="n">
-        <v>100.881759072301</v>
-      </c>
-      <c r="C7" s="7" t="n">
-        <v>100.888331097064</v>
-      </c>
-      <c r="D7" s="7" t="n">
-        <v>100.574713990694</v>
-      </c>
-      <c r="E7" s="7" t="n">
-        <v>101.20292613999</v>
-      </c>
-      <c r="F7" s="7" t="n">
-        <v>103.881661770877</v>
-      </c>
-      <c r="G7" s="7" t="n">
-        <v>104.003980856891</v>
-      </c>
-      <c r="H7" s="7" t="n">
-        <v>103.528256830621</v>
-      </c>
-      <c r="I7" s="7" t="n">
-        <v>104.48189088876</v>
-      </c>
-      <c r="J7" s="6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="12" t="n">
-        <v>44986</v>
-      </c>
-      <c r="B8" s="7" t="n">
-        <v>101.090158012708</v>
-      </c>
-      <c r="C8" s="7" t="n">
-        <v>100.850993578064</v>
-      </c>
-      <c r="D8" s="7" t="n">
-        <v>100.55059409583</v>
-      </c>
-      <c r="E8" s="7" t="n">
-        <v>101.15229051744</v>
-      </c>
-      <c r="F8" s="7" t="n">
-        <v>103.75863121352</v>
-      </c>
-      <c r="G8" s="7" t="n">
-        <v>103.833229467584</v>
-      </c>
-      <c r="H8" s="7" t="n">
-        <v>103.378120878282</v>
-      </c>
-      <c r="I8" s="7" t="n">
-        <v>104.290341612632</v>
-      </c>
-      <c r="J8" s="6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="12" t="n">
-        <v>45017</v>
-      </c>
-      <c r="B9" s="7" t="n">
-        <v>101.164255413741</v>
-      </c>
-      <c r="C9" s="7" t="n">
-        <v>100.809671728626</v>
-      </c>
-      <c r="D9" s="7" t="n">
-        <v>100.523896673753</v>
-      </c>
-      <c r="E9" s="7" t="n">
-        <v>101.096259201089</v>
-      </c>
-      <c r="F9" s="7" t="n">
-        <v>103.796780223553</v>
-      </c>
-      <c r="G9" s="7" t="n">
-        <v>103.644510266199</v>
-      </c>
-      <c r="H9" s="7" t="n">
-        <v>103.212152885396</v>
-      </c>
-      <c r="I9" s="7" t="n">
-        <v>104.078678799077</v>
-      </c>
-      <c r="J9" s="6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="12" t="n">
-        <v>45047</v>
-      </c>
-      <c r="B10" s="7" t="n">
-        <v>101.470833410518</v>
-      </c>
-      <c r="C10" s="7" t="n">
-        <v>100.769698962589</v>
-      </c>
-      <c r="D10" s="7" t="n">
-        <v>100.49806720805</v>
-      </c>
-      <c r="E10" s="7" t="n">
-        <v>101.042064898511</v>
-      </c>
-      <c r="F10" s="7" t="n">
-        <v>103.950329988937</v>
-      </c>
-      <c r="G10" s="7" t="n">
-        <v>103.462205370336</v>
-      </c>
-      <c r="H10" s="7" t="n">
-        <v>103.05179240153</v>
-      </c>
-      <c r="I10" s="7" t="n">
-        <v>103.874252845453</v>
-      </c>
-      <c r="J10" s="6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="12" t="n">
-        <v>45078</v>
-      </c>
-      <c r="B11" s="7" t="n">
-        <v>101.292073430524</v>
-      </c>
-      <c r="C11" s="7" t="n">
-        <v>100.728410422132</v>
-      </c>
-      <c r="D11" s="7" t="n">
-        <v>100.471383732509</v>
-      </c>
-      <c r="E11" s="7" t="n">
-        <v>100.986094639468</v>
-      </c>
-      <c r="F11" s="7" t="n">
-        <v>103.561210086598</v>
-      </c>
-      <c r="G11" s="7" t="n">
-        <v>103.274160513491</v>
-      </c>
-      <c r="H11" s="7" t="n">
-        <v>102.886348311398</v>
-      </c>
-      <c r="I11" s="7" t="n">
-        <v>103.663434506255</v>
-      </c>
-      <c r="J11" s="6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="12" t="n">
-        <v>45108</v>
-      </c>
-      <c r="B12" s="7" t="n">
-        <v>100.842857936758</v>
-      </c>
-      <c r="C12" s="7" t="n">
-        <v>100.688469877599</v>
-      </c>
-      <c r="D12" s="7" t="n">
-        <v>100.445567759929</v>
-      </c>
-      <c r="E12" s="7" t="n">
-        <v>100.931959392404</v>
-      </c>
-      <c r="F12" s="7" t="n">
-        <v>102.872620455499</v>
-      </c>
-      <c r="G12" s="7" t="n">
-        <v>103.092507042126</v>
-      </c>
-      <c r="H12" s="7" t="n">
-        <v>102.726494029347</v>
-      </c>
-      <c r="I12" s="7" t="n">
-        <v>103.459824153977</v>
-      </c>
-      <c r="J12" s="6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="12" t="n">
-        <v>45139</v>
-      </c>
-      <c r="B13" s="7" t="n">
-        <v>100.77061297075</v>
-      </c>
-      <c r="C13" s="7" t="n">
-        <v>100.647214619273</v>
-      </c>
-      <c r="D13" s="7" t="n">
-        <v>100.418898223638</v>
-      </c>
-      <c r="E13" s="7" t="n">
-        <v>100.876050124134</v>
-      </c>
-      <c r="F13" s="7" t="n">
-        <v>102.497806431923</v>
-      </c>
-      <c r="G13" s="7" t="n">
-        <v>102.905134120206</v>
-      </c>
-      <c r="H13" s="7" t="n">
-        <v>102.561572188193</v>
-      </c>
-      <c r="I13" s="7" t="n">
-        <v>103.249846919923</v>
-      </c>
-      <c r="J13" s="6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="12" t="n">
-        <v>45170</v>
-      </c>
-      <c r="B14" s="7" t="n">
-        <v>100.673360131893</v>
-      </c>
-      <c r="C14" s="7" t="n">
-        <v>100.605976264535</v>
-      </c>
-      <c r="D14" s="7" t="n">
-        <v>100.392235768438</v>
-      </c>
-      <c r="E14" s="7" t="n">
-        <v>100.820171825701</v>
-      </c>
-      <c r="F14" s="7" t="n">
-        <v>102.374775874566</v>
-      </c>
-      <c r="G14" s="7" t="n">
-        <v>102.718101752734</v>
-      </c>
-      <c r="H14" s="7" t="n">
-        <v>102.396915120153</v>
-      </c>
-      <c r="I14" s="7" t="n">
-        <v>103.04029584587</v>
-      </c>
-      <c r="J14" s="6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="12" t="n">
-        <v>45200</v>
-      </c>
-      <c r="B15" s="7" t="n">
-        <v>100.833595761629</v>
-      </c>
-      <c r="C15" s="7" t="n">
-        <v>100.566084267248</v>
-      </c>
-      <c r="D15" s="7" t="n">
-        <v>100.366440132809</v>
-      </c>
-      <c r="E15" s="7" t="n">
-        <v>100.766125524275</v>
-      </c>
-      <c r="F15" s="7" t="n">
-        <v>102.245069240453</v>
-      </c>
-      <c r="G15" s="7" t="n">
-        <v>102.537426357625</v>
-      </c>
-      <c r="H15" s="7" t="n">
-        <v>102.237821269323</v>
-      </c>
-      <c r="I15" s="7" t="n">
-        <v>102.837909430295</v>
-      </c>
-      <c r="J15" s="6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="12" t="n">
-        <v>45231</v>
-      </c>
-      <c r="B16" s="7" t="n">
-        <v>100.462182538947</v>
-      </c>
-      <c r="C16" s="7" t="n">
-        <v>100.524879154187</v>
-      </c>
-      <c r="D16" s="7" t="n">
-        <v>100.339791605879</v>
-      </c>
-      <c r="E16" s="7" t="n">
-        <v>100.710308116405</v>
-      </c>
-      <c r="F16" s="7" t="n">
-        <v>101.723381528249</v>
-      </c>
-      <c r="G16" s="7" t="n">
-        <v>102.35106230718</v>
-      </c>
-      <c r="H16" s="7" t="n">
-        <v>102.073683965907</v>
-      </c>
-      <c r="I16" s="7" t="n">
-        <v>102.62919440536</v>
-      </c>
-      <c r="J16" s="6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="12" t="n">
-        <v>45261</v>
-      </c>
-      <c r="B17" s="7" t="n">
-        <v>100.203767852843</v>
-      </c>
-      <c r="C17" s="7" t="n">
-        <v>100.485019313297</v>
-      </c>
-      <c r="D17" s="7" t="n">
-        <v>100.314009445699</v>
-      </c>
-      <c r="E17" s="7" t="n">
-        <v>100.656320709216</v>
-      </c>
-      <c r="F17" s="7" t="n">
-        <v>101.281806737115</v>
-      </c>
-      <c r="G17" s="7" t="n">
-        <v>102.171032513924</v>
-      </c>
-      <c r="H17" s="7" t="n">
-        <v>101.915092318575</v>
-      </c>
-      <c r="I17" s="7" t="n">
-        <v>102.427615453955</v>
-      </c>
-      <c r="J17" s="6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="12" t="n">
-        <v>45292</v>
-      </c>
-      <c r="B18" s="7" t="n">
-        <v>100.166719152326</v>
-      </c>
-      <c r="C18" s="7" t="n">
-        <v>100.443847415118</v>
-      </c>
-      <c r="D18" s="7" t="n">
-        <v>100.287374839763</v>
-      </c>
-      <c r="E18" s="7" t="n">
-        <v>100.600564125559</v>
-      </c>
-      <c r="F18" s="7" t="n">
-        <v>101.477320413535</v>
-      </c>
-      <c r="G18" s="7" t="n">
-        <v>101.985334392431</v>
-      </c>
-      <c r="H18" s="7" t="n">
-        <v>101.75147313907</v>
-      </c>
-      <c r="I18" s="7" t="n">
-        <v>102.219733142539</v>
-      </c>
-      <c r="J18" s="6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="12" t="n">
-        <v>45323</v>
-      </c>
-      <c r="B19" s="7" t="n">
-        <v>100.481633106719</v>
-      </c>
-      <c r="C19" s="7" t="n">
-        <v>100.402692386371</v>
-      </c>
-      <c r="D19" s="7" t="n">
-        <v>100.260747305643</v>
-      </c>
-      <c r="E19" s="7" t="n">
-        <v>100.544838427161</v>
-      </c>
-      <c r="F19" s="7" t="n">
-        <v>101.730057605005</v>
-      </c>
-      <c r="G19" s="7" t="n">
-        <v>101.799973781399</v>
-      </c>
-      <c r="H19" s="7" t="n">
-        <v>101.588116641325</v>
-      </c>
-      <c r="I19" s="7" t="n">
-        <v>102.012272739368</v>
-      </c>
-      <c r="J19" s="6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="12" t="n">
-        <v>45352</v>
-      </c>
-      <c r="B20" s="7" t="n">
-        <v>100.585369468166</v>
-      </c>
-      <c r="C20" s="7" t="n">
-        <v>100.364207786661</v>
-      </c>
-      <c r="D20" s="7" t="n">
-        <v>100.235844077451</v>
-      </c>
-      <c r="E20" s="7" t="n">
-        <v>100.492735880597</v>
-      </c>
-      <c r="F20" s="7" t="n">
-        <v>101.819707778583</v>
-      </c>
-      <c r="G20" s="7" t="n">
-        <v>101.626876926622</v>
-      </c>
-      <c r="H20" s="7" t="n">
-        <v>101.43553670651</v>
-      </c>
-      <c r="I20" s="7" t="n">
-        <v>101.818578076256</v>
-      </c>
-      <c r="J20" s="6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="12" t="n">
-        <v>45383</v>
-      </c>
-      <c r="B21" s="7" t="n">
-        <v>100.640942518941</v>
-      </c>
-      <c r="C21" s="7" t="n">
-        <v>100.323085388794</v>
-      </c>
-      <c r="D21" s="7" t="n">
-        <v>100.209230225383</v>
-      </c>
-      <c r="E21" s="7" t="n">
-        <v>100.437069911529</v>
-      </c>
-      <c r="F21" s="7" t="n">
-        <v>101.599397245641</v>
-      </c>
-      <c r="G21" s="7" t="n">
-        <v>101.442167819998</v>
-      </c>
-      <c r="H21" s="7" t="n">
-        <v>101.272687427654</v>
-      </c>
-      <c r="I21" s="7" t="n">
-        <v>101.611931838698</v>
-      </c>
-      <c r="J21" s="6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="12" t="n">
-        <v>45413</v>
-      </c>
-      <c r="B22" s="7" t="n">
-        <v>100.43439601356</v>
-      </c>
-      <c r="C22" s="7" t="n">
-        <v>100.283305562597</v>
-      </c>
-      <c r="D22" s="7" t="n">
-        <v>100.183481612756</v>
-      </c>
-      <c r="E22" s="7" t="n">
-        <v>100.383228978147</v>
-      </c>
-      <c r="F22" s="7" t="n">
-        <v>100.716247663373</v>
-      </c>
-      <c r="G22" s="7" t="n">
-        <v>101.263736721302</v>
-      </c>
-      <c r="H22" s="7" t="n">
-        <v>101.115340286796</v>
-      </c>
-      <c r="I22" s="7" t="n">
-        <v>101.412350941772</v>
-      </c>
-      <c r="J22" s="6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="12" t="n">
-        <v>45444</v>
-      </c>
-      <c r="B23" s="7" t="n">
-        <v>100.486264194283</v>
-      </c>
-      <c r="C23" s="7" t="n">
-        <v>100.242216312937</v>
-      </c>
-      <c r="D23" s="7" t="n">
-        <v>100.156881663568</v>
-      </c>
-      <c r="E23" s="7" t="n">
-        <v>100.327623668268</v>
-      </c>
-      <c r="F23" s="7" t="n">
-        <v>100.663792774577</v>
-      </c>
-      <c r="G23" s="7" t="n">
-        <v>101.079687630069</v>
-      </c>
-      <c r="H23" s="7" t="n">
-        <v>100.953005066008</v>
-      </c>
-      <c r="I23" s="7" t="n">
-        <v>101.206529163861</v>
-      </c>
-      <c r="J23" s="6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="12" t="n">
-        <v>45474</v>
-      </c>
-      <c r="B24" s="7" t="n">
-        <v>100.425133838431</v>
-      </c>
-      <c r="C24" s="7" t="n">
-        <v>100.202468552718</v>
-      </c>
-      <c r="D24" s="7" t="n">
-        <v>100.131146501826</v>
-      </c>
-      <c r="E24" s="7" t="n">
-        <v>100.273841405334</v>
-      </c>
-      <c r="F24" s="7" t="n">
-        <v>100.440621065883</v>
-      </c>
-      <c r="G24" s="7" t="n">
-        <v>100.901894113752</v>
-      </c>
-      <c r="H24" s="7" t="n">
-        <v>100.796154614898</v>
-      </c>
-      <c r="I24" s="7" t="n">
-        <v>101.007744537884</v>
-      </c>
-      <c r="J24" s="6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="12" t="n">
-        <v>45505</v>
-      </c>
-      <c r="B25" s="7" t="n">
-        <v>100.295463386622</v>
-      </c>
-      <c r="C25" s="7" t="n">
-        <v>100.161412424543</v>
-      </c>
-      <c r="D25" s="7" t="n">
-        <v>100.104560448255</v>
-      </c>
-      <c r="E25" s="7" t="n">
-        <v>100.218296688544</v>
-      </c>
-      <c r="F25" s="7" t="n">
-        <v>100.297562278259</v>
-      </c>
-      <c r="G25" s="7" t="n">
-        <v>100.718502679497</v>
-      </c>
-      <c r="H25" s="7" t="n">
-        <v>100.634331829478</v>
-      </c>
-      <c r="I25" s="7" t="n">
-        <v>100.802743930261</v>
-      </c>
-      <c r="J25" s="6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="12" t="n">
-        <v>45536</v>
-      </c>
-      <c r="B26" s="7" t="n">
-        <v>100.337143174703</v>
-      </c>
-      <c r="C26" s="7" t="n">
-        <v>100.120373118366</v>
-      </c>
-      <c r="D26" s="7" t="n">
-        <v>100.077981453609</v>
-      </c>
-      <c r="E26" s="7" t="n">
-        <v>100.162782739653</v>
-      </c>
-      <c r="F26" s="7" t="n">
-        <v>100.508335558692</v>
-      </c>
-      <c r="G26" s="7" t="n">
-        <v>100.535444563248</v>
-      </c>
-      <c r="H26" s="7" t="n">
-        <v>100.472768841804</v>
-      </c>
-      <c r="I26" s="7" t="n">
-        <v>100.598159382311</v>
-      </c>
-      <c r="J26" s="6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="12" t="n">
-        <v>45566</v>
-      </c>
-      <c r="B27" s="7" t="n">
-        <v>100.397347313043</v>
-      </c>
-      <c r="C27" s="7" t="n">
-        <v>100.080673671066</v>
-      </c>
-      <c r="D27" s="7" t="n">
-        <v>100.052266565158</v>
-      </c>
-      <c r="E27" s="7" t="n">
-        <v>100.109088842394</v>
-      </c>
-      <c r="F27" s="7" t="n">
-        <v>100.548392019227</v>
-      </c>
-      <c r="G27" s="7" t="n">
-        <v>100.358608340041</v>
-      </c>
-      <c r="H27" s="7" t="n">
-        <v>100.316664532608</v>
-      </c>
-      <c r="I27" s="7" t="n">
-        <v>100.400569684769</v>
-      </c>
-      <c r="J27" s="6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="12" t="n">
-        <v>45597</v>
-      </c>
-      <c r="B28" s="7" t="n">
-        <v>100.27601281885</v>
-      </c>
-      <c r="C28" s="7" t="n">
-        <v>100.039667446116</v>
-      </c>
-      <c r="D28" s="7" t="n">
-        <v>100.025701455183</v>
-      </c>
-      <c r="E28" s="7" t="n">
-        <v>100.053635387036</v>
-      </c>
-      <c r="F28" s="7" t="n">
-        <v>100.488307328425</v>
-      </c>
-      <c r="G28" s="7" t="n">
-        <v>100.176204339749</v>
-      </c>
-      <c r="H28" s="7" t="n">
-        <v>100.155611542632</v>
-      </c>
-      <c r="I28" s="7" t="n">
-        <v>100.196801370911</v>
-      </c>
-      <c r="J28" s="6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="12" t="n">
-        <v>45627</v>
-      </c>
-      <c r="B29" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="C29" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="D29" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="E29" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="F29" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="G29" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="H29" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="I29" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="J29" s="6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="12" t="n">
-        <v>45658</v>
-      </c>
-      <c r="B30" s="7" t="n">
-        <v>100.399199748069</v>
-      </c>
-      <c r="C30" s="7" t="n">
-        <v>99.9590268296107</v>
-      </c>
-      <c r="D30" s="7" t="n">
-        <v>99.944606972255</v>
-      </c>
-      <c r="E30" s="7" t="n">
-        <v>99.9734487674418</v>
-      </c>
-      <c r="F30" s="7" t="n">
-        <v>100.308053256018</v>
-      </c>
-      <c r="G30" s="7" t="n">
-        <v>99.8182477783339</v>
-      </c>
-      <c r="H30" s="7" t="n">
-        <v>99.797044663693</v>
-      </c>
-      <c r="I30" s="7" t="n">
-        <v>99.8394553978384</v>
-      </c>
-      <c r="J30" s="6" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="12" t="n">
-        <v>45689</v>
-      </c>
-      <c r="B31" s="7" t="n">
-        <v>100.813218976344</v>
-      </c>
-      <c r="C31" s="7" t="n">
-        <v>99.9180704472284</v>
-      </c>
-      <c r="D31" s="7" t="n">
-        <v>99.8892446283852</v>
-      </c>
-      <c r="E31" s="7" t="n">
-        <v>99.946904584563</v>
-      </c>
-      <c r="F31" s="7" t="n">
-        <v>100.715293938122</v>
-      </c>
-      <c r="G31" s="7" t="n">
-        <v>99.6368258953686</v>
-      </c>
-      <c r="H31" s="7" t="n">
-        <v>99.5945012360713</v>
-      </c>
-      <c r="I31" s="7" t="n">
-        <v>99.6791685413697</v>
-      </c>
-      <c r="J31" s="6" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="12" t="n">
-        <v>45717</v>
-      </c>
-      <c r="B32" s="7" t="n">
-        <v>100.548320767649</v>
-      </c>
-      <c r="C32" s="7" t="n">
-        <v>99.8810920096502</v>
-      </c>
-      <c r="D32" s="7" t="n">
-        <v>99.8392662900037</v>
-      </c>
-      <c r="E32" s="7" t="n">
-        <v>99.9229352513688</v>
-      </c>
-      <c r="F32" s="7" t="n">
-        <v>100.665700225079</v>
-      </c>
-      <c r="G32" s="7" t="n">
-        <v>99.4732444025496</v>
-      </c>
-      <c r="H32" s="7" t="n">
-        <v>99.4119121342112</v>
-      </c>
-      <c r="I32" s="7" t="n">
-        <v>99.5346145098859</v>
-      </c>
-      <c r="J32" s="6" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="12" t="n">
-        <v>45748</v>
-      </c>
-      <c r="B33" s="7" t="n">
-        <v>100.83730063168</v>
-      </c>
-      <c r="C33" s="7" t="n">
-        <v>99.8401675596344</v>
-      </c>
-      <c r="D33" s="7" t="n">
-        <v>99.7839622975272</v>
-      </c>
-      <c r="E33" s="7" t="n">
-        <v>99.8964044804512</v>
-      </c>
-      <c r="F33" s="7" t="n">
-        <v>101.157822454507</v>
-      </c>
-      <c r="G33" s="7" t="n">
-        <v>99.2924495708846</v>
-      </c>
-      <c r="H33" s="7" t="n">
-        <v>99.21015035361</v>
-      </c>
-      <c r="I33" s="7" t="n">
-        <v>99.374817059008</v>
-      </c>
-      <c r="J33" s="6" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="12" t="n">
-        <v>45778</v>
-      </c>
-      <c r="B34" s="7" t="n">
-        <v>101.086453142656</v>
-      </c>
-      <c r="C34" s="7" t="n">
-        <v>99.8005792186497</v>
-      </c>
-      <c r="D34" s="7" t="n">
-        <v>99.7304714731594</v>
-      </c>
-      <c r="E34" s="7" t="n">
-        <v>99.8707362479337</v>
-      </c>
-      <c r="F34" s="7" t="n">
-        <v>101.178804410026</v>
-      </c>
-      <c r="G34" s="7" t="n">
-        <v>99.1177997063379</v>
-      </c>
-      <c r="H34" s="7" t="n">
-        <v>99.0152869115566</v>
-      </c>
-      <c r="I34" s="7" t="n">
-        <v>99.220418634964</v>
-      </c>
-      <c r="J34" s="6" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="12" t="n">
-        <v>45809</v>
-      </c>
-      <c r="B35" s="7" t="n">
-        <v>101.484726673212</v>
-      </c>
-      <c r="C35" s="7" t="n">
-        <v>99.759687757277</v>
-      </c>
-      <c r="D35" s="7" t="n">
-        <v>99.6752277454261</v>
-      </c>
-      <c r="E35" s="7" t="n">
-        <v>99.8442193364949</v>
-      </c>
-      <c r="F35" s="7" t="n">
-        <v>101.657574485942</v>
-      </c>
-      <c r="G35" s="7" t="n">
-        <v>98.9376509033051</v>
-      </c>
-      <c r="H35" s="7" t="n">
-        <v>98.8143301030099</v>
-      </c>
-      <c r="I35" s="7" t="n">
-        <v>99.0611256086035</v>
-      </c>
-      <c r="J35" s="6" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="12" t="n">
-        <v>45839</v>
-      </c>
-      <c r="B36" s="7" t="n">
-        <v>101.483800455699</v>
-      </c>
-      <c r="C36" s="7" t="n">
-        <v>99.7201313279161</v>
-      </c>
-      <c r="D36" s="7" t="n">
-        <v>99.6217952099926</v>
-      </c>
-      <c r="E36" s="7" t="n">
-        <v>99.8185645128726</v>
-      </c>
-      <c r="F36" s="7" t="n">
-        <v>101.533590203334</v>
-      </c>
-      <c r="G36" s="7" t="n">
-        <v>98.7636251097678</v>
-      </c>
-      <c r="H36" s="7" t="n">
-        <v>98.6202441106044</v>
-      </c>
-      <c r="I36" s="7" t="n">
-        <v>98.9072145662425</v>
-      </c>
-      <c r="J36" s="6" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="12" t="n">
-        <v>45870</v>
-      </c>
-      <c r="B37" s="7" t="n">
-        <v>101.36987570161</v>
-      </c>
-      <c r="C37" s="7" t="n">
-        <v>99.6792728285947</v>
-      </c>
-      <c r="D37" s="7" t="n">
-        <v>99.5666116813319</v>
-      </c>
-      <c r="E37" s="7" t="n">
-        <v>99.7920614536725</v>
-      </c>
-      <c r="F37" s="7" t="n">
-        <v>101.451569831763</v>
-      </c>
-      <c r="G37" s="7" t="n">
-        <v>98.5841200269329</v>
-      </c>
-      <c r="H37" s="7" t="n">
-        <v>98.420089062503</v>
-      </c>
-      <c r="I37" s="7" t="n">
-        <v>98.748424372108</v>
-      </c>
-      <c r="J37" s="6" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="12" t="n">
-        <v>45901</v>
-      </c>
-      <c r="B38" s="7" t="n">
-        <v>101.548635681603</v>
-      </c>
-      <c r="C38" s="7" t="n">
-        <v>99.6384310702958</v>
-      </c>
-      <c r="D38" s="7" t="n">
-        <v>99.5114587204985</v>
-      </c>
-      <c r="E38" s="7" t="n">
-        <v>99.7655654313613</v>
-      </c>
-      <c r="F38" s="7" t="n">
-        <v>101.386716514706</v>
-      </c>
-      <c r="G38" s="7" t="n">
-        <v>98.404941198574</v>
-      </c>
-      <c r="H38" s="7" t="n">
-        <v>98.2203402397525</v>
-      </c>
-      <c r="I38" s="7" t="n">
-        <v>98.589889107059</v>
-      </c>
-      <c r="J38" s="6" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="12" t="n">
-        <v>45931</v>
-      </c>
-      <c r="B39" s="7" t="n">
-        <v>101.545857029065</v>
-      </c>
-      <c r="C39" s="7" t="n">
-        <v>99.5989227212936</v>
-      </c>
-      <c r="D39" s="7" t="n">
-        <v>99.4581139761283</v>
-      </c>
-      <c r="E39" s="7" t="n">
-        <v>99.7399308177428</v>
-      </c>
-      <c r="F39" s="7" t="n">
-        <v>101.46015335902</v>
-      </c>
-      <c r="G39" s="7" t="n">
-        <v>98.2318524116085</v>
-      </c>
-      <c r="H39" s="7" t="n">
-        <v>98.0274209314906</v>
-      </c>
-      <c r="I39" s="7" t="n">
-        <v>98.4367102237635</v>
-      </c>
-      <c r="J39" s="6" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="12" t="n">
-        <v>45962</v>
-      </c>
-      <c r="B40" s="7" t="n">
-        <v>101.52548024378</v>
-      </c>
-      <c r="C40" s="7" t="n">
-        <v>99.5581138849812</v>
-      </c>
-      <c r="D40" s="7" t="n">
-        <v>99.4030211154588</v>
-      </c>
-      <c r="E40" s="7" t="n">
-        <v>99.713448636758</v>
-      </c>
-      <c r="F40" s="7" t="n">
-        <v>101.495441193301</v>
-      </c>
-      <c r="G40" s="7" t="n">
-        <v>98.0533138374666</v>
-      </c>
-      <c r="H40" s="7" t="n">
-        <v>97.828469049666</v>
-      </c>
-      <c r="I40" s="7" t="n">
-        <v>98.2786753989538</v>
-      </c>
-      <c r="J40" s="6" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="12" t="n">
-        <v>45992</v>
-      </c>
-      <c r="B41" s="7" t="n">
-        <v>101.966359779931</v>
-      </c>
-      <c r="C41" s="7" t="n">
-        <v>99.5186373831222</v>
-      </c>
-      <c r="D41" s="7" t="n">
-        <v>99.3497345008397</v>
-      </c>
-      <c r="E41" s="7" t="n">
-        <v>99.6878274144724</v>
-      </c>
-      <c r="F41" s="7" t="n">
-        <v>102.051463014535</v>
-      </c>
-      <c r="G41" s="7" t="n">
-        <v>97.8808435433599</v>
-      </c>
-      <c r="H41" s="7" t="n">
-        <v>97.6363194345118</v>
-      </c>
-      <c r="I41" s="7" t="n">
-        <v>98.1259800476787</v>
-      </c>
-      <c r="J41" s="6" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="13" t="n">
-        <v>46023</v>
-      </c>
-      <c r="B42" s="11" t="n">
-        <v>102.271085341682</v>
-      </c>
-      <c r="C42" s="11" t="n">
-        <v>99.4778614422581</v>
-      </c>
-      <c r="D42" s="11" t="n">
-        <v>99.2947016748431</v>
-      </c>
-      <c r="E42" s="11" t="n">
-        <v>99.6613590675834</v>
-      </c>
-      <c r="F42" s="11" t="n">
-        <v>102.472055850151</v>
-      </c>
-      <c r="G42" s="11" t="n">
-        <v>97.7029429356343</v>
-      </c>
-      <c r="H42" s="11" t="n">
-        <v>97.4381613140457</v>
-      </c>
-      <c r="I42" s="11" t="n">
-        <v>97.968444083394</v>
-      </c>
-      <c r="J42" s="10" t="b">
-        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -31852,24 +31486,26 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="83.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="11.71" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="80.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="12.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="13.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="26.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="29.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>70</v>
+        <v>202</v>
       </c>
     </row>
     <row r="5">
@@ -31877,10 +31513,16 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>82</v>
+        <v>203</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>83</v>
+        <v>204</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="6">
@@ -31888,10 +31530,16 @@
         <v>45627</v>
       </c>
       <c r="B6" s="7" t="n">
-        <v>0</v>
+        <v>253703</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>0</v>
+        <v>243438.774684143</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>11.7687358107597</v>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>11.7687358107597</v>
       </c>
     </row>
     <row r="7">
@@ -31899,10 +31547,16 @@
         <v>45658</v>
       </c>
       <c r="B7" s="7" t="n">
-        <v>0.440353345184574</v>
+        <v>285683</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>0.490697330984813</v>
+        <v>244374.646013476</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>47.3632534248561</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>59.1319892356158</v>
       </c>
     </row>
     <row r="8">
@@ -31910,10 +31564,16 @@
         <v>45689</v>
       </c>
       <c r="B8" s="7" t="n">
-        <v>0.895882521659397</v>
+        <v>282954</v>
       </c>
       <c r="C8" s="7" t="n">
-        <v>1.08239903576031</v>
+        <v>245310.517342808</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>43.1611922728362</v>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>102.293181508452</v>
       </c>
     </row>
     <row r="9">
@@ -31921,10 +31581,16 @@
         <v>45717</v>
       </c>
       <c r="B9" s="7" t="n">
-        <v>0.668023090831293</v>
+        <v>300358</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>1.19877041277943</v>
+        <v>246155.820478979</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>62.1470312196687</v>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>164.440212728121</v>
       </c>
     </row>
     <row r="10">
@@ -31932,10 +31598,16 @@
         <v>45748</v>
       </c>
       <c r="B10" s="7" t="n">
-        <v>0.9987293655636</v>
+        <v>240461</v>
       </c>
       <c r="C10" s="7" t="n">
-        <v>1.87866538864165</v>
+        <v>247091.691808312</v>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>-7.60260591844516</v>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>156.837606809676</v>
       </c>
     </row>
     <row r="11">
@@ -31943,10 +31615,16 @@
         <v>45778</v>
       </c>
       <c r="B11" s="7" t="n">
-        <v>1.28844334779772</v>
+        <v>241089</v>
       </c>
       <c r="C11" s="7" t="n">
-        <v>2.07934872423914</v>
+        <v>247997.373739924</v>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>-7.92098993594275</v>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>148.916616873733</v>
       </c>
     </row>
     <row r="12">
@@ -31954,10 +31632,16 @@
         <v>45809</v>
       </c>
       <c r="B12" s="7" t="n">
-        <v>1.72919438173473</v>
+        <v>230650</v>
       </c>
       <c r="C12" s="7" t="n">
-        <v>2.74912892898098</v>
+        <v>248933.245069256</v>
+      </c>
+      <c r="D12" s="7" t="n">
+        <v>-20.9631681263894</v>
+      </c>
+      <c r="E12" s="7" t="n">
+        <v>127.953448747343</v>
       </c>
     </row>
     <row r="13">
@@ -31965,10 +31649,16 @@
         <v>45839</v>
       </c>
       <c r="B13" s="7" t="n">
-        <v>1.76861893811928</v>
+        <v>245921</v>
       </c>
       <c r="C13" s="7" t="n">
-        <v>2.80464097028412</v>
+        <v>249838.927000868</v>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>-4.49220923938841</v>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>123.461239507955</v>
       </c>
     </row>
     <row r="14">
@@ -31976,10 +31666,16 @@
         <v>45870</v>
       </c>
       <c r="B14" s="7" t="n">
-        <v>1.69604254228677</v>
+        <v>229128</v>
       </c>
       <c r="C14" s="7" t="n">
-        <v>2.9086325506041</v>
+        <v>250774.7983302</v>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>-24.8197445844608</v>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>98.6414949234942</v>
       </c>
     </row>
     <row r="15">
@@ -31987,10 +31683,16 @@
         <v>45901</v>
       </c>
       <c r="B15" s="7" t="n">
-        <v>1.91713638080069</v>
+        <v>231589</v>
       </c>
       <c r="C15" s="7" t="n">
-        <v>3.03010730946474</v>
+        <v>251710.669659533</v>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>-23.0710654732595</v>
+      </c>
+      <c r="E15" s="7" t="n">
+        <v>75.5704294502347</v>
       </c>
     </row>
     <row r="16">
@@ -31998,10 +31700,16 @@
         <v>45931</v>
       </c>
       <c r="B16" s="7" t="n">
-        <v>1.95477446399612</v>
+        <v>221136</v>
       </c>
       <c r="C16" s="7" t="n">
-        <v>3.28640951804993</v>
+        <v>252616.351591145</v>
+      </c>
+      <c r="D16" s="7" t="n">
+        <v>-36.0946812550641</v>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>39.4757481951706</v>
       </c>
     </row>
     <row r="17">
@@ -32009,10 +31717,16 @@
         <v>45962</v>
       </c>
       <c r="B17" s="7" t="n">
-        <v>1.97609846352873</v>
+        <v>233624</v>
       </c>
       <c r="C17" s="7" t="n">
-        <v>3.51046509406108</v>
+        <v>253552.222920477</v>
+      </c>
+      <c r="D17" s="7" t="n">
+        <v>-22.8492636815663</v>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>16.6264845136043</v>
       </c>
     </row>
     <row r="18">
@@ -32020,10 +31734,16 @@
         <v>45992</v>
       </c>
       <c r="B18" s="7" t="n">
-        <v>2.45956180789071</v>
+        <v>242150</v>
       </c>
       <c r="C18" s="7" t="n">
-        <v>4.26091492491825</v>
+        <v>254457.904852089</v>
+      </c>
+      <c r="D18" s="7" t="n">
+        <v>-14.111973980582</v>
+      </c>
+      <c r="E18" s="7" t="n">
+        <v>2.51451053302223</v>
       </c>
     </row>
     <row r="19">
@@ -32031,10 +31751,16 @@
         <v>46023</v>
       </c>
       <c r="B19" s="11" t="n">
-        <v>2.80788494940138</v>
+        <v>238920</v>
       </c>
       <c r="C19" s="11" t="n">
-        <v>4.88123773063647</v>
+        <v>255393.776181421</v>
+      </c>
+      <c r="D19" s="11" t="n">
+        <v>-18.8884707533868</v>
+      </c>
+      <c r="E19" s="11" t="n">
+        <v>-16.3739602203646</v>
       </c>
     </row>
   </sheetData>
@@ -32048,27 +31774,1477 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
+    <col min="1" max="1" width="86.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="16.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="29.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="29.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="29.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="19.71" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="32.71" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="32.71" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="32.71" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="18.71" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="n">
+        <v>44927</v>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>100.693736917178</v>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>100.92968518895</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>100.601424908979</v>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>101.259016575136</v>
+      </c>
+      <c r="F6" s="7" t="n">
+        <v>103.849235112349</v>
+      </c>
+      <c r="G6" s="7" t="n">
+        <v>104.193354593693</v>
+      </c>
+      <c r="H6" s="7" t="n">
+        <v>103.694733127383</v>
+      </c>
+      <c r="I6" s="7" t="n">
+        <v>104.694373707011</v>
+      </c>
+      <c r="J6" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="n">
+        <v>44958</v>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>100.881759072301</v>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>100.888331097064</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>100.574713990694</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>101.20292613999</v>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>103.881661770877</v>
+      </c>
+      <c r="G7" s="7" t="n">
+        <v>104.003980856891</v>
+      </c>
+      <c r="H7" s="7" t="n">
+        <v>103.528256830621</v>
+      </c>
+      <c r="I7" s="7" t="n">
+        <v>104.48189088876</v>
+      </c>
+      <c r="J7" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="n">
+        <v>44986</v>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>101.090158012708</v>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>100.850993578064</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>100.55059409583</v>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>101.15229051744</v>
+      </c>
+      <c r="F8" s="7" t="n">
+        <v>103.75863121352</v>
+      </c>
+      <c r="G8" s="7" t="n">
+        <v>103.833229467584</v>
+      </c>
+      <c r="H8" s="7" t="n">
+        <v>103.378120878282</v>
+      </c>
+      <c r="I8" s="7" t="n">
+        <v>104.290341612632</v>
+      </c>
+      <c r="J8" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="n">
+        <v>45017</v>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>101.164255413741</v>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>100.809671728626</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>100.523896673753</v>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>101.096259201089</v>
+      </c>
+      <c r="F9" s="7" t="n">
+        <v>103.796780223553</v>
+      </c>
+      <c r="G9" s="7" t="n">
+        <v>103.644510266199</v>
+      </c>
+      <c r="H9" s="7" t="n">
+        <v>103.212152885396</v>
+      </c>
+      <c r="I9" s="7" t="n">
+        <v>104.078678799077</v>
+      </c>
+      <c r="J9" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="n">
+        <v>45047</v>
+      </c>
+      <c r="B10" s="7" t="n">
+        <v>101.470833410518</v>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>100.769698962589</v>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>100.49806720805</v>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>101.042064898511</v>
+      </c>
+      <c r="F10" s="7" t="n">
+        <v>103.950329988937</v>
+      </c>
+      <c r="G10" s="7" t="n">
+        <v>103.462205370336</v>
+      </c>
+      <c r="H10" s="7" t="n">
+        <v>103.05179240153</v>
+      </c>
+      <c r="I10" s="7" t="n">
+        <v>103.874252845453</v>
+      </c>
+      <c r="J10" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="n">
+        <v>45078</v>
+      </c>
+      <c r="B11" s="7" t="n">
+        <v>101.292073430524</v>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>100.728410422132</v>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>100.471383732509</v>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>100.986094639468</v>
+      </c>
+      <c r="F11" s="7" t="n">
+        <v>103.561210086598</v>
+      </c>
+      <c r="G11" s="7" t="n">
+        <v>103.274160513491</v>
+      </c>
+      <c r="H11" s="7" t="n">
+        <v>102.886348311398</v>
+      </c>
+      <c r="I11" s="7" t="n">
+        <v>103.663434506255</v>
+      </c>
+      <c r="J11" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="n">
+        <v>45108</v>
+      </c>
+      <c r="B12" s="7" t="n">
+        <v>100.842857936758</v>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>100.688469877599</v>
+      </c>
+      <c r="D12" s="7" t="n">
+        <v>100.445567759929</v>
+      </c>
+      <c r="E12" s="7" t="n">
+        <v>100.931959392404</v>
+      </c>
+      <c r="F12" s="7" t="n">
+        <v>102.872620455499</v>
+      </c>
+      <c r="G12" s="7" t="n">
+        <v>103.092507042126</v>
+      </c>
+      <c r="H12" s="7" t="n">
+        <v>102.726494029347</v>
+      </c>
+      <c r="I12" s="7" t="n">
+        <v>103.459824153977</v>
+      </c>
+      <c r="J12" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="n">
+        <v>45139</v>
+      </c>
+      <c r="B13" s="7" t="n">
+        <v>100.77061297075</v>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>100.647214619273</v>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>100.418898223638</v>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>100.876050124134</v>
+      </c>
+      <c r="F13" s="7" t="n">
+        <v>102.497806431923</v>
+      </c>
+      <c r="G13" s="7" t="n">
+        <v>102.905134120206</v>
+      </c>
+      <c r="H13" s="7" t="n">
+        <v>102.561572188193</v>
+      </c>
+      <c r="I13" s="7" t="n">
+        <v>103.249846919923</v>
+      </c>
+      <c r="J13" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="n">
+        <v>45170</v>
+      </c>
+      <c r="B14" s="7" t="n">
+        <v>100.673360131893</v>
+      </c>
+      <c r="C14" s="7" t="n">
+        <v>100.605976264535</v>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>100.392235768438</v>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>100.820171825701</v>
+      </c>
+      <c r="F14" s="7" t="n">
+        <v>102.374775874566</v>
+      </c>
+      <c r="G14" s="7" t="n">
+        <v>102.718101752734</v>
+      </c>
+      <c r="H14" s="7" t="n">
+        <v>102.396915120153</v>
+      </c>
+      <c r="I14" s="7" t="n">
+        <v>103.04029584587</v>
+      </c>
+      <c r="J14" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="n">
+        <v>45200</v>
+      </c>
+      <c r="B15" s="7" t="n">
+        <v>100.833595761629</v>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>100.566084267248</v>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>100.366440132809</v>
+      </c>
+      <c r="E15" s="7" t="n">
+        <v>100.766125524275</v>
+      </c>
+      <c r="F15" s="7" t="n">
+        <v>102.245069240453</v>
+      </c>
+      <c r="G15" s="7" t="n">
+        <v>102.537426357625</v>
+      </c>
+      <c r="H15" s="7" t="n">
+        <v>102.237821269323</v>
+      </c>
+      <c r="I15" s="7" t="n">
+        <v>102.837909430295</v>
+      </c>
+      <c r="J15" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="n">
+        <v>45231</v>
+      </c>
+      <c r="B16" s="7" t="n">
+        <v>100.462182538947</v>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>100.524879154187</v>
+      </c>
+      <c r="D16" s="7" t="n">
+        <v>100.339791605879</v>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>100.710308116405</v>
+      </c>
+      <c r="F16" s="7" t="n">
+        <v>101.723381528249</v>
+      </c>
+      <c r="G16" s="7" t="n">
+        <v>102.35106230718</v>
+      </c>
+      <c r="H16" s="7" t="n">
+        <v>102.073683965907</v>
+      </c>
+      <c r="I16" s="7" t="n">
+        <v>102.62919440536</v>
+      </c>
+      <c r="J16" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="n">
+        <v>45261</v>
+      </c>
+      <c r="B17" s="7" t="n">
+        <v>100.203767852843</v>
+      </c>
+      <c r="C17" s="7" t="n">
+        <v>100.485019313297</v>
+      </c>
+      <c r="D17" s="7" t="n">
+        <v>100.314009445699</v>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>100.656320709216</v>
+      </c>
+      <c r="F17" s="7" t="n">
+        <v>101.281806737115</v>
+      </c>
+      <c r="G17" s="7" t="n">
+        <v>102.171032513924</v>
+      </c>
+      <c r="H17" s="7" t="n">
+        <v>101.915092318575</v>
+      </c>
+      <c r="I17" s="7" t="n">
+        <v>102.427615453955</v>
+      </c>
+      <c r="J17" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="n">
+        <v>45292</v>
+      </c>
+      <c r="B18" s="7" t="n">
+        <v>100.166719152326</v>
+      </c>
+      <c r="C18" s="7" t="n">
+        <v>100.443847415118</v>
+      </c>
+      <c r="D18" s="7" t="n">
+        <v>100.287374839763</v>
+      </c>
+      <c r="E18" s="7" t="n">
+        <v>100.600564125559</v>
+      </c>
+      <c r="F18" s="7" t="n">
+        <v>101.477320413535</v>
+      </c>
+      <c r="G18" s="7" t="n">
+        <v>101.985334392431</v>
+      </c>
+      <c r="H18" s="7" t="n">
+        <v>101.75147313907</v>
+      </c>
+      <c r="I18" s="7" t="n">
+        <v>102.219733142539</v>
+      </c>
+      <c r="J18" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="n">
+        <v>45323</v>
+      </c>
+      <c r="B19" s="7" t="n">
+        <v>100.481633106719</v>
+      </c>
+      <c r="C19" s="7" t="n">
+        <v>100.402692386371</v>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>100.260747305643</v>
+      </c>
+      <c r="E19" s="7" t="n">
+        <v>100.544838427161</v>
+      </c>
+      <c r="F19" s="7" t="n">
+        <v>101.730057605005</v>
+      </c>
+      <c r="G19" s="7" t="n">
+        <v>101.799973781399</v>
+      </c>
+      <c r="H19" s="7" t="n">
+        <v>101.588116641325</v>
+      </c>
+      <c r="I19" s="7" t="n">
+        <v>102.012272739368</v>
+      </c>
+      <c r="J19" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="n">
+        <v>45352</v>
+      </c>
+      <c r="B20" s="7" t="n">
+        <v>100.585369468166</v>
+      </c>
+      <c r="C20" s="7" t="n">
+        <v>100.364207786661</v>
+      </c>
+      <c r="D20" s="7" t="n">
+        <v>100.235844077451</v>
+      </c>
+      <c r="E20" s="7" t="n">
+        <v>100.492735880597</v>
+      </c>
+      <c r="F20" s="7" t="n">
+        <v>101.819707778583</v>
+      </c>
+      <c r="G20" s="7" t="n">
+        <v>101.626876926622</v>
+      </c>
+      <c r="H20" s="7" t="n">
+        <v>101.43553670651</v>
+      </c>
+      <c r="I20" s="7" t="n">
+        <v>101.818578076256</v>
+      </c>
+      <c r="J20" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="n">
+        <v>45383</v>
+      </c>
+      <c r="B21" s="7" t="n">
+        <v>100.640942518941</v>
+      </c>
+      <c r="C21" s="7" t="n">
+        <v>100.323085388794</v>
+      </c>
+      <c r="D21" s="7" t="n">
+        <v>100.209230225383</v>
+      </c>
+      <c r="E21" s="7" t="n">
+        <v>100.437069911529</v>
+      </c>
+      <c r="F21" s="7" t="n">
+        <v>101.599397245641</v>
+      </c>
+      <c r="G21" s="7" t="n">
+        <v>101.442167819998</v>
+      </c>
+      <c r="H21" s="7" t="n">
+        <v>101.272687427654</v>
+      </c>
+      <c r="I21" s="7" t="n">
+        <v>101.611931838698</v>
+      </c>
+      <c r="J21" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="n">
+        <v>45413</v>
+      </c>
+      <c r="B22" s="7" t="n">
+        <v>100.43439601356</v>
+      </c>
+      <c r="C22" s="7" t="n">
+        <v>100.283305562597</v>
+      </c>
+      <c r="D22" s="7" t="n">
+        <v>100.183481612756</v>
+      </c>
+      <c r="E22" s="7" t="n">
+        <v>100.383228978147</v>
+      </c>
+      <c r="F22" s="7" t="n">
+        <v>100.716247663373</v>
+      </c>
+      <c r="G22" s="7" t="n">
+        <v>101.263736721302</v>
+      </c>
+      <c r="H22" s="7" t="n">
+        <v>101.115340286796</v>
+      </c>
+      <c r="I22" s="7" t="n">
+        <v>101.412350941772</v>
+      </c>
+      <c r="J22" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="n">
+        <v>45444</v>
+      </c>
+      <c r="B23" s="7" t="n">
+        <v>100.486264194283</v>
+      </c>
+      <c r="C23" s="7" t="n">
+        <v>100.242216312937</v>
+      </c>
+      <c r="D23" s="7" t="n">
+        <v>100.156881663568</v>
+      </c>
+      <c r="E23" s="7" t="n">
+        <v>100.327623668268</v>
+      </c>
+      <c r="F23" s="7" t="n">
+        <v>100.663792774577</v>
+      </c>
+      <c r="G23" s="7" t="n">
+        <v>101.079687630069</v>
+      </c>
+      <c r="H23" s="7" t="n">
+        <v>100.953005066008</v>
+      </c>
+      <c r="I23" s="7" t="n">
+        <v>101.206529163861</v>
+      </c>
+      <c r="J23" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="n">
+        <v>45474</v>
+      </c>
+      <c r="B24" s="7" t="n">
+        <v>100.425133838431</v>
+      </c>
+      <c r="C24" s="7" t="n">
+        <v>100.202468552718</v>
+      </c>
+      <c r="D24" s="7" t="n">
+        <v>100.131146501826</v>
+      </c>
+      <c r="E24" s="7" t="n">
+        <v>100.273841405334</v>
+      </c>
+      <c r="F24" s="7" t="n">
+        <v>100.440621065883</v>
+      </c>
+      <c r="G24" s="7" t="n">
+        <v>100.901894113752</v>
+      </c>
+      <c r="H24" s="7" t="n">
+        <v>100.796154614898</v>
+      </c>
+      <c r="I24" s="7" t="n">
+        <v>101.007744537884</v>
+      </c>
+      <c r="J24" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="n">
+        <v>45505</v>
+      </c>
+      <c r="B25" s="7" t="n">
+        <v>100.295463386622</v>
+      </c>
+      <c r="C25" s="7" t="n">
+        <v>100.161412424543</v>
+      </c>
+      <c r="D25" s="7" t="n">
+        <v>100.104560448255</v>
+      </c>
+      <c r="E25" s="7" t="n">
+        <v>100.218296688544</v>
+      </c>
+      <c r="F25" s="7" t="n">
+        <v>100.297562278259</v>
+      </c>
+      <c r="G25" s="7" t="n">
+        <v>100.718502679497</v>
+      </c>
+      <c r="H25" s="7" t="n">
+        <v>100.634331829478</v>
+      </c>
+      <c r="I25" s="7" t="n">
+        <v>100.802743930261</v>
+      </c>
+      <c r="J25" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="n">
+        <v>45536</v>
+      </c>
+      <c r="B26" s="7" t="n">
+        <v>100.337143174703</v>
+      </c>
+      <c r="C26" s="7" t="n">
+        <v>100.120373118366</v>
+      </c>
+      <c r="D26" s="7" t="n">
+        <v>100.077981453609</v>
+      </c>
+      <c r="E26" s="7" t="n">
+        <v>100.162782739653</v>
+      </c>
+      <c r="F26" s="7" t="n">
+        <v>100.508335558692</v>
+      </c>
+      <c r="G26" s="7" t="n">
+        <v>100.535444563248</v>
+      </c>
+      <c r="H26" s="7" t="n">
+        <v>100.472768841804</v>
+      </c>
+      <c r="I26" s="7" t="n">
+        <v>100.598159382311</v>
+      </c>
+      <c r="J26" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="n">
+        <v>45566</v>
+      </c>
+      <c r="B27" s="7" t="n">
+        <v>100.397347313043</v>
+      </c>
+      <c r="C27" s="7" t="n">
+        <v>100.080673671066</v>
+      </c>
+      <c r="D27" s="7" t="n">
+        <v>100.052266565158</v>
+      </c>
+      <c r="E27" s="7" t="n">
+        <v>100.109088842394</v>
+      </c>
+      <c r="F27" s="7" t="n">
+        <v>100.548392019227</v>
+      </c>
+      <c r="G27" s="7" t="n">
+        <v>100.358608340041</v>
+      </c>
+      <c r="H27" s="7" t="n">
+        <v>100.316664532608</v>
+      </c>
+      <c r="I27" s="7" t="n">
+        <v>100.400569684769</v>
+      </c>
+      <c r="J27" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="n">
+        <v>45597</v>
+      </c>
+      <c r="B28" s="7" t="n">
+        <v>100.27601281885</v>
+      </c>
+      <c r="C28" s="7" t="n">
+        <v>100.039667446116</v>
+      </c>
+      <c r="D28" s="7" t="n">
+        <v>100.025701455183</v>
+      </c>
+      <c r="E28" s="7" t="n">
+        <v>100.053635387036</v>
+      </c>
+      <c r="F28" s="7" t="n">
+        <v>100.488307328425</v>
+      </c>
+      <c r="G28" s="7" t="n">
+        <v>100.176204339749</v>
+      </c>
+      <c r="H28" s="7" t="n">
+        <v>100.155611542632</v>
+      </c>
+      <c r="I28" s="7" t="n">
+        <v>100.196801370911</v>
+      </c>
+      <c r="J28" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="12" t="n">
+        <v>45627</v>
+      </c>
+      <c r="B29" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="C29" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="D29" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="E29" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="F29" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="G29" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="H29" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="I29" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J29" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="12" t="n">
+        <v>45658</v>
+      </c>
+      <c r="B30" s="7" t="n">
+        <v>100.399199748069</v>
+      </c>
+      <c r="C30" s="7" t="n">
+        <v>99.9590268296107</v>
+      </c>
+      <c r="D30" s="7" t="n">
+        <v>99.944606972255</v>
+      </c>
+      <c r="E30" s="7" t="n">
+        <v>99.9734487674418</v>
+      </c>
+      <c r="F30" s="7" t="n">
+        <v>100.308053256018</v>
+      </c>
+      <c r="G30" s="7" t="n">
+        <v>99.8182477783339</v>
+      </c>
+      <c r="H30" s="7" t="n">
+        <v>99.797044663693</v>
+      </c>
+      <c r="I30" s="7" t="n">
+        <v>99.8394553978384</v>
+      </c>
+      <c r="J30" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="n">
+        <v>45689</v>
+      </c>
+      <c r="B31" s="7" t="n">
+        <v>100.813218976344</v>
+      </c>
+      <c r="C31" s="7" t="n">
+        <v>99.9180704472284</v>
+      </c>
+      <c r="D31" s="7" t="n">
+        <v>99.8892446283852</v>
+      </c>
+      <c r="E31" s="7" t="n">
+        <v>99.946904584563</v>
+      </c>
+      <c r="F31" s="7" t="n">
+        <v>100.715293938122</v>
+      </c>
+      <c r="G31" s="7" t="n">
+        <v>99.6368258953686</v>
+      </c>
+      <c r="H31" s="7" t="n">
+        <v>99.5945012360713</v>
+      </c>
+      <c r="I31" s="7" t="n">
+        <v>99.6791685413697</v>
+      </c>
+      <c r="J31" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="n">
+        <v>45717</v>
+      </c>
+      <c r="B32" s="7" t="n">
+        <v>100.548320767649</v>
+      </c>
+      <c r="C32" s="7" t="n">
+        <v>99.8810920096502</v>
+      </c>
+      <c r="D32" s="7" t="n">
+        <v>99.8392662900037</v>
+      </c>
+      <c r="E32" s="7" t="n">
+        <v>99.9229352513688</v>
+      </c>
+      <c r="F32" s="7" t="n">
+        <v>100.665700225079</v>
+      </c>
+      <c r="G32" s="7" t="n">
+        <v>99.4732444025496</v>
+      </c>
+      <c r="H32" s="7" t="n">
+        <v>99.4119121342112</v>
+      </c>
+      <c r="I32" s="7" t="n">
+        <v>99.5346145098859</v>
+      </c>
+      <c r="J32" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="12" t="n">
+        <v>45748</v>
+      </c>
+      <c r="B33" s="7" t="n">
+        <v>100.83730063168</v>
+      </c>
+      <c r="C33" s="7" t="n">
+        <v>99.8401675596344</v>
+      </c>
+      <c r="D33" s="7" t="n">
+        <v>99.7839622975272</v>
+      </c>
+      <c r="E33" s="7" t="n">
+        <v>99.8964044804512</v>
+      </c>
+      <c r="F33" s="7" t="n">
+        <v>101.157822454507</v>
+      </c>
+      <c r="G33" s="7" t="n">
+        <v>99.2924495708846</v>
+      </c>
+      <c r="H33" s="7" t="n">
+        <v>99.21015035361</v>
+      </c>
+      <c r="I33" s="7" t="n">
+        <v>99.374817059008</v>
+      </c>
+      <c r="J33" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="12" t="n">
+        <v>45778</v>
+      </c>
+      <c r="B34" s="7" t="n">
+        <v>101.086453142656</v>
+      </c>
+      <c r="C34" s="7" t="n">
+        <v>99.8005792186497</v>
+      </c>
+      <c r="D34" s="7" t="n">
+        <v>99.7304714731594</v>
+      </c>
+      <c r="E34" s="7" t="n">
+        <v>99.8707362479337</v>
+      </c>
+      <c r="F34" s="7" t="n">
+        <v>101.178804410026</v>
+      </c>
+      <c r="G34" s="7" t="n">
+        <v>99.1177997063379</v>
+      </c>
+      <c r="H34" s="7" t="n">
+        <v>99.0152869115566</v>
+      </c>
+      <c r="I34" s="7" t="n">
+        <v>99.220418634964</v>
+      </c>
+      <c r="J34" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="n">
+        <v>45809</v>
+      </c>
+      <c r="B35" s="7" t="n">
+        <v>101.484726673212</v>
+      </c>
+      <c r="C35" s="7" t="n">
+        <v>99.759687757277</v>
+      </c>
+      <c r="D35" s="7" t="n">
+        <v>99.6752277454261</v>
+      </c>
+      <c r="E35" s="7" t="n">
+        <v>99.8442193364949</v>
+      </c>
+      <c r="F35" s="7" t="n">
+        <v>101.657574485942</v>
+      </c>
+      <c r="G35" s="7" t="n">
+        <v>98.9376509033051</v>
+      </c>
+      <c r="H35" s="7" t="n">
+        <v>98.8143301030099</v>
+      </c>
+      <c r="I35" s="7" t="n">
+        <v>99.0611256086035</v>
+      </c>
+      <c r="J35" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="12" t="n">
+        <v>45839</v>
+      </c>
+      <c r="B36" s="7" t="n">
+        <v>101.483800455699</v>
+      </c>
+      <c r="C36" s="7" t="n">
+        <v>99.7201313279161</v>
+      </c>
+      <c r="D36" s="7" t="n">
+        <v>99.6217952099926</v>
+      </c>
+      <c r="E36" s="7" t="n">
+        <v>99.8185645128726</v>
+      </c>
+      <c r="F36" s="7" t="n">
+        <v>101.533590203334</v>
+      </c>
+      <c r="G36" s="7" t="n">
+        <v>98.7636251097678</v>
+      </c>
+      <c r="H36" s="7" t="n">
+        <v>98.6202441106044</v>
+      </c>
+      <c r="I36" s="7" t="n">
+        <v>98.9072145662425</v>
+      </c>
+      <c r="J36" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="12" t="n">
+        <v>45870</v>
+      </c>
+      <c r="B37" s="7" t="n">
+        <v>101.36987570161</v>
+      </c>
+      <c r="C37" s="7" t="n">
+        <v>99.6792728285947</v>
+      </c>
+      <c r="D37" s="7" t="n">
+        <v>99.5666116813319</v>
+      </c>
+      <c r="E37" s="7" t="n">
+        <v>99.7920614536725</v>
+      </c>
+      <c r="F37" s="7" t="n">
+        <v>101.451569831763</v>
+      </c>
+      <c r="G37" s="7" t="n">
+        <v>98.5841200269329</v>
+      </c>
+      <c r="H37" s="7" t="n">
+        <v>98.420089062503</v>
+      </c>
+      <c r="I37" s="7" t="n">
+        <v>98.748424372108</v>
+      </c>
+      <c r="J37" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="12" t="n">
+        <v>45901</v>
+      </c>
+      <c r="B38" s="7" t="n">
+        <v>101.548635681603</v>
+      </c>
+      <c r="C38" s="7" t="n">
+        <v>99.6384310702958</v>
+      </c>
+      <c r="D38" s="7" t="n">
+        <v>99.5114587204985</v>
+      </c>
+      <c r="E38" s="7" t="n">
+        <v>99.7655654313613</v>
+      </c>
+      <c r="F38" s="7" t="n">
+        <v>101.386716514706</v>
+      </c>
+      <c r="G38" s="7" t="n">
+        <v>98.404941198574</v>
+      </c>
+      <c r="H38" s="7" t="n">
+        <v>98.2203402397525</v>
+      </c>
+      <c r="I38" s="7" t="n">
+        <v>98.589889107059</v>
+      </c>
+      <c r="J38" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="12" t="n">
+        <v>45931</v>
+      </c>
+      <c r="B39" s="7" t="n">
+        <v>101.545857029065</v>
+      </c>
+      <c r="C39" s="7" t="n">
+        <v>99.5989227212936</v>
+      </c>
+      <c r="D39" s="7" t="n">
+        <v>99.4581139761283</v>
+      </c>
+      <c r="E39" s="7" t="n">
+        <v>99.7399308177428</v>
+      </c>
+      <c r="F39" s="7" t="n">
+        <v>101.46015335902</v>
+      </c>
+      <c r="G39" s="7" t="n">
+        <v>98.2318524116085</v>
+      </c>
+      <c r="H39" s="7" t="n">
+        <v>98.0274209314906</v>
+      </c>
+      <c r="I39" s="7" t="n">
+        <v>98.4367102237635</v>
+      </c>
+      <c r="J39" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="12" t="n">
+        <v>45962</v>
+      </c>
+      <c r="B40" s="7" t="n">
+        <v>101.52548024378</v>
+      </c>
+      <c r="C40" s="7" t="n">
+        <v>99.5581138849812</v>
+      </c>
+      <c r="D40" s="7" t="n">
+        <v>99.4030211154588</v>
+      </c>
+      <c r="E40" s="7" t="n">
+        <v>99.713448636758</v>
+      </c>
+      <c r="F40" s="7" t="n">
+        <v>101.495441193301</v>
+      </c>
+      <c r="G40" s="7" t="n">
+        <v>98.0533138374666</v>
+      </c>
+      <c r="H40" s="7" t="n">
+        <v>97.828469049666</v>
+      </c>
+      <c r="I40" s="7" t="n">
+        <v>98.2786753989538</v>
+      </c>
+      <c r="J40" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="12" t="n">
+        <v>45992</v>
+      </c>
+      <c r="B41" s="7" t="n">
+        <v>101.966359779931</v>
+      </c>
+      <c r="C41" s="7" t="n">
+        <v>99.5186373831222</v>
+      </c>
+      <c r="D41" s="7" t="n">
+        <v>99.3497345008397</v>
+      </c>
+      <c r="E41" s="7" t="n">
+        <v>99.6878274144724</v>
+      </c>
+      <c r="F41" s="7" t="n">
+        <v>102.051463014535</v>
+      </c>
+      <c r="G41" s="7" t="n">
+        <v>97.8808435433599</v>
+      </c>
+      <c r="H41" s="7" t="n">
+        <v>97.6363194345118</v>
+      </c>
+      <c r="I41" s="7" t="n">
+        <v>98.1259800476787</v>
+      </c>
+      <c r="J41" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="13" t="n">
+        <v>46023</v>
+      </c>
+      <c r="B42" s="11" t="n">
+        <v>102.271085341682</v>
+      </c>
+      <c r="C42" s="11" t="n">
+        <v>99.4778614422581</v>
+      </c>
+      <c r="D42" s="11" t="n">
+        <v>99.2947016748431</v>
+      </c>
+      <c r="E42" s="11" t="n">
+        <v>99.6613590675834</v>
+      </c>
+      <c r="F42" s="11" t="n">
+        <v>102.472055850151</v>
+      </c>
+      <c r="G42" s="11" t="n">
+        <v>97.7029429356343</v>
+      </c>
+      <c r="H42" s="11" t="n">
+        <v>97.4381613140457</v>
+      </c>
+      <c r="I42" s="11" t="n">
+        <v>97.968444083394</v>
+      </c>
+      <c r="J42" s="10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="83.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="11.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="13.71" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="n">
+        <v>45627</v>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="n">
+        <v>45658</v>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>0.440353345184574</v>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>0.490697330984813</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="n">
+        <v>45689</v>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>0.895882521659397</v>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>1.08239903576031</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="n">
+        <v>45717</v>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>0.668023090831293</v>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>1.19877041277943</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="n">
+        <v>45748</v>
+      </c>
+      <c r="B10" s="7" t="n">
+        <v>0.9987293655636</v>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>1.87866538864165</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="n">
+        <v>45778</v>
+      </c>
+      <c r="B11" s="7" t="n">
+        <v>1.28844334779772</v>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>2.07934872423914</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="n">
+        <v>45809</v>
+      </c>
+      <c r="B12" s="7" t="n">
+        <v>1.72919438173473</v>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>2.74912892898098</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="n">
+        <v>45839</v>
+      </c>
+      <c r="B13" s="7" t="n">
+        <v>1.76861893811928</v>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>2.80464097028412</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="n">
+        <v>45870</v>
+      </c>
+      <c r="B14" s="7" t="n">
+        <v>1.69604254228677</v>
+      </c>
+      <c r="C14" s="7" t="n">
+        <v>2.9086325506041</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="n">
+        <v>45901</v>
+      </c>
+      <c r="B15" s="7" t="n">
+        <v>1.91713638080069</v>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>3.03010730946474</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="n">
+        <v>45931</v>
+      </c>
+      <c r="B16" s="7" t="n">
+        <v>1.95477446399612</v>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>3.28640951804993</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="n">
+        <v>45962</v>
+      </c>
+      <c r="B17" s="7" t="n">
+        <v>1.97609846352873</v>
+      </c>
+      <c r="C17" s="7" t="n">
+        <v>3.51046509406108</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="n">
+        <v>45992</v>
+      </c>
+      <c r="B18" s="7" t="n">
+        <v>2.45956180789071</v>
+      </c>
+      <c r="C18" s="7" t="n">
+        <v>4.26091492491825</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="n">
+        <v>46023</v>
+      </c>
+      <c r="B19" s="11" t="n">
+        <v>2.80788494940138</v>
+      </c>
+      <c r="C19" s="11" t="n">
+        <v>4.88123773063647</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
     <col min="1" max="1" width="80.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
     </row>
     <row r="6">
@@ -32138,36 +33314,46 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="str">
-        <f>HYPERLINK("#'F11'!A1", "Figure 11. Manufacturing Industrial Production")</f>
+        <f>HYPERLINK("#'F9'!A1", "Figure 9. Tariff-Exposed Employment Index")</f>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="str">
-        <f>HYPERLINK("#'F12'!A1", "Figure 12. Nominal Effective Exchange Rates (Daily)")</f>
+        <f>HYPERLINK("#'F10'!A1", "Figure 10. Manufacturing Tariff-Exposed Employment Index")</f>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="str">
-        <f>HYPERLINK("#'F13'!A1", "Figure 13. Real US Imports and Exports")</f>
+        <f>HYPERLINK("#'F11'!A1", "Figure 11. Manufacturing Industrial Production")</f>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="str">
-        <f>HYPERLINK("#'F14'!A1", "Figure 14. Trade Deviation from Trend")</f>
+        <f>HYPERLINK("#'F12'!A1", "Figure 12. Nominal Effective Exchange Rates (Daily)")</f>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="str">
-        <f>HYPERLINK("#'F15'!A1", "Figure 15. Cumulative Import Gap vs. Trend")</f>
+        <f>HYPERLINK("#'F13'!A1", "Figure 13. Real US Imports and Exports")</f>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="str">
-        <f>HYPERLINK("#'FA2'!A1", "Figure A2. PCE Core Goods &amp; Durables Prices (Log-Linear Trend)")</f>
+        <f>HYPERLINK("#'F14'!A1", "Figure 14. Trade Deviation from Trend")</f>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="str">
+        <f>HYPERLINK("#'F15'!A1", "Figure 15. Cumulative Import Gap vs. Trend")</f>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="str">
+        <f>HYPERLINK("#'FA2'!A1", "Figure A2. PCE Core Goods &amp; Durables Prices (Log-Linear Trend)")</f>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="str">
         <f>HYPERLINK("#'FA3'!A1", "Figure A3. PCE Goods Prices: Deviation from Log-Linear Trend")</f>
       </c>
     </row>

</xml_diff>